<commit_message>
Checklist RCP: todas las preguntas con lista de respuestas posibles; solo la contraseña se escribe
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vbz2Sf1pkMwtP6vBTAs1UZ
</commit_message>
<xml_diff>
--- a/RCP_Checklist_Recepcion_Tecnica.xlsx
+++ b/RCP_Checklist_Recepcion_Tecnica.xlsx
@@ -16,12 +16,34 @@
     <definedName name="T_EQUIPO">Listas!$A$2:$A$5</definedName>
     <definedName name="L_YN">Listas!$C$2:$C$3</definedName>
     <definedName name="L_YNS">Listas!$D$2:$D$4</definedName>
-    <definedName name="L_CUANDO">Listas!$T$2:$T$6</definedName>
-    <definedName name="L_MOM">Listas!$U$2:$U$5</definedName>
-    <definedName name="L_LIQ">Listas!$V$2:$V$8</definedName>
-    <definedName name="L_E_PANT">Listas!$W$2:$W$5</definedName>
-    <definedName name="L_E_CARC">Listas!$X$2:$X$5</definedName>
-    <definedName name="L_PIN">Listas!$Y$2:$Y$5</definedName>
+    <definedName name="L_YNC">Listas!$T$2:$T$4</definedName>
+    <definedName name="L_FUN">Listas!$U$2:$U$4</definedName>
+    <definedName name="L_FALLAP">Listas!$V$2:$V$12</definedName>
+    <definedName name="L_DESDE">Listas!$W$2:$W$8</definedName>
+    <definedName name="L_PERM">Listas!$X$2:$X$4</definedName>
+    <definedName name="L_ENC">Listas!$Y$2:$Y$5</definedName>
+    <definedName name="L_OTRAF">Listas!$Z$2:$Z$10</definedName>
+    <definedName name="L_LUZ">Listas!$AA$2:$AA$8</definedName>
+    <definedName name="L_SENAL">Listas!$AB$2:$AB$6</definedName>
+    <definedName name="L_AUTON">Listas!$AC$2:$AC$7</definedName>
+    <definedName name="L_ZONAC">Listas!$AD$2:$AD$7</definedName>
+    <definedName name="L_MANT">Listas!$AE$2:$AE$6</definedName>
+    <definedName name="L_ABCE">Listas!$AF$2:$AF$4</definedName>
+    <definedName name="L_ZONAI">Listas!$AG$2:$AG$9</definedName>
+    <definedName name="L_ERR">Listas!$AH$2:$AH$7</definedName>
+    <definedName name="L_PROG">Listas!$AI$2:$AI$8</definedName>
+    <definedName name="L_SO">Listas!$AJ$2:$AJ$7</definedName>
+    <definedName name="L_TEL">Listas!$AK$2:$AK$4</definedName>
+    <definedName name="L_JUE">Listas!$AL$2:$AL$5</definedName>
+    <definedName name="L_NCTRL">Listas!$AM$2:$AM$5</definedName>
+    <definedName name="L_SOL">Listas!$AN$2:$AN$8</definedName>
+    <definedName name="L_DANO">Listas!$AO$2:$AO$8</definedName>
+    <definedName name="L_CUANDO">Listas!$AP$2:$AP$6</definedName>
+    <definedName name="L_MOM">Listas!$AQ$2:$AQ$5</definedName>
+    <definedName name="L_LIQ">Listas!$AR$2:$AR$8</definedName>
+    <definedName name="L_E_PANT">Listas!$AS$2:$AS$5</definedName>
+    <definedName name="L_E_CARC">Listas!$AT$2:$AT$5</definedName>
+    <definedName name="L_PIN">Listas!$AU$2:$AU$5</definedName>
     <definedName name="F_Celular">Listas!$F$2:$F$12</definedName>
     <definedName name="F_Reloj">Listas!$G$2:$G$12</definedName>
     <definedName name="F_Computadora">Listas!$H$2:$H$14</definedName>
@@ -732,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C17"/>
+  <dimension ref="B1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -798,7 +820,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Cada fila es una pregunta. Las de Sí/No tienen lista desplegable y se pintan de color; las que piden un dato (falla, fecha, tipo de líquido, estado de pantalla) tienen su propia lista o se escriben directamente en la respuesta. Use «Detalle» para notas.</t>
+          <t>Cada fila es una pregunta. Las de Sí/No tienen lista desplegable y se pintan de color; las que piden un dato (falla, fecha, tipo de líquido, estado de pantalla…) tienen su propia lista de opciones. Nada se escribe, excepto la contraseña/PIN y las notas opcionales de «Detalle».</t>
         </is>
       </c>
     </row>
@@ -881,32 +903,44 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="2" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Contraseña</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Es la única respuesta que se escribe a mano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>PERSONALIZAR</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="B16" s="3" t="inlineStr">
+    <row r="17" ht="32" customHeight="1">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Banco_Preguntas</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Contiene todas las preguntas. Puede editar textos o agregar preguntas al final indicando bloque, tipo (YN, YNS, TXT) y marcando 1/0 los equipos donde aplica.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="3" t="inlineStr">
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Importante</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Abra el archivo en Excel. Las vistas previas no recalculan y no mostrarán el cambio automático.</t>
         </is>
@@ -916,8 +950,8 @@
   <mergeCells count="4">
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B15:C15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5261,13 +5295,13 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="D24:D193">
     <cfRule type="expression" priority="5" dxfId="4" stopIfTrue="1">
-      <formula>$D24="Sí"</formula>
+      <formula>OR($D24="Sí",$D24="Funciona")</formula>
     </cfRule>
     <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
-      <formula>$D24="No"</formula>
+      <formula>OR($D24="No",$D24="No funciona")</formula>
     </cfRule>
     <cfRule type="expression" priority="7" dxfId="5" stopIfTrue="1">
-      <formula>$D24="No sé"</formula>
+      <formula>OR($D24="No sé",$D24="No probado",$D24="No fue posible comprobar")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D24:E193">
@@ -5377,7 +5411,7 @@
       </c>
       <c r="M1" s="23" t="inlineStr">
         <is>
-          <t>Cómo editar: agregue una pregunta al final. Sección B = según la falla (escriba el Bloque exacto); S = siempre para ese equipo. Tipo: YN = Sí/No · YNS = Sí/No/No sé · TXT = texto libre · CUANDO, MOM, LIQ, E_PANT, E_CARC, PIN = lista de opciones (hoja Listas) · HEAD = título. Marque 1/0 en los equipos donde aplica. Las columnas grises se calculan solas.</t>
+          <t>Cómo editar: agregue una pregunta al final. Sección B = según la falla (escriba el Bloque exacto); S = siempre para ese equipo. Tipo: YN = Sí/No (los demás tipos son listas de la hoja Listas: escriba el nombre sin «L_») · YNS = Sí/No/No sé · TXT = texto libre · CUANDO, MOM, LIQ, E_PANT, E_CARC, PIN = lista de opciones (hoja Listas) · HEAD = título. Marque 1/0 en los equipos donde aplica. Las columnas grises se calculan solas.</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5475,7 @@
       </c>
       <c r="D3" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>FALLAP</t>
         </is>
       </c>
       <c r="E3" s="26" t="n">
@@ -5487,7 +5521,7 @@
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>DESDE</t>
         </is>
       </c>
       <c r="E4" s="26" t="n">
@@ -5528,12 +5562,12 @@
       </c>
       <c r="C5" s="25" t="inlineStr">
         <is>
-          <t>¿La falla es permanente? (No = sucede algunas veces)</t>
+          <t>¿La falla es permanente o sucede algunas veces?</t>
         </is>
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>PERM</t>
         </is>
       </c>
       <c r="E5" s="26" t="n">
@@ -5579,7 +5613,7 @@
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E6" s="26" t="n">
@@ -5625,7 +5659,7 @@
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E7" s="26" t="n">
@@ -5717,7 +5751,7 @@
       </c>
       <c r="D9" s="24" t="inlineStr">
         <is>
-          <t>YNS</t>
+          <t>ENC</t>
         </is>
       </c>
       <c r="E9" s="26" t="n">
@@ -5758,12 +5792,12 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>¿Enciende solo de forma intermitente?</t>
+          <t>¿El equipo se reinicia o se apaga solo?</t>
         </is>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E10" s="26" t="n">
@@ -5809,7 +5843,7 @@
       </c>
       <c r="D11" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E11" s="26" t="n">
@@ -5901,7 +5935,7 @@
       </c>
       <c r="D13" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>OTRAF</t>
         </is>
       </c>
       <c r="E13" s="26" t="n">
@@ -6035,7 +6069,7 @@
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E16" s="26" t="n">
@@ -6081,7 +6115,7 @@
       </c>
       <c r="D17" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E17" s="26" t="n">
@@ -6127,7 +6161,7 @@
       </c>
       <c r="D18" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>SENAL</t>
         </is>
       </c>
       <c r="E18" s="26" t="n">
@@ -6173,7 +6207,7 @@
       </c>
       <c r="D19" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E19" s="26" t="n">
@@ -6219,7 +6253,7 @@
       </c>
       <c r="D20" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E20" s="26" t="n">
@@ -6265,7 +6299,7 @@
       </c>
       <c r="D21" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E21" s="26" t="n">
@@ -6311,7 +6345,7 @@
       </c>
       <c r="D22" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E22" s="26" t="n">
@@ -6357,7 +6391,7 @@
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E23" s="26" t="n">
@@ -6403,7 +6437,7 @@
       </c>
       <c r="D24" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>LUZ</t>
         </is>
       </c>
       <c r="E24" s="26" t="n">
@@ -6449,7 +6483,7 @@
       </c>
       <c r="D25" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E25" s="26" t="n">
@@ -6495,7 +6529,7 @@
       </c>
       <c r="D26" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E26" s="26" t="n">
@@ -6541,7 +6575,7 @@
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E27" s="26" t="n">
@@ -6587,7 +6621,7 @@
       </c>
       <c r="D28" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E28" s="26" t="n">
@@ -6633,7 +6667,7 @@
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E29" s="26" t="n">
@@ -6679,7 +6713,7 @@
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E30" s="26" t="n">
@@ -6725,7 +6759,7 @@
       </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E31" s="26" t="n">
@@ -6771,7 +6805,7 @@
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E32" s="26" t="n">
@@ -6817,7 +6851,7 @@
       </c>
       <c r="D33" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E33" s="26" t="n">
@@ -6863,7 +6897,7 @@
       </c>
       <c r="D34" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E34" s="26" t="n">
@@ -6909,7 +6943,7 @@
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E35" s="26" t="n">
@@ -6955,7 +6989,7 @@
       </c>
       <c r="D36" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E36" s="26" t="n">
@@ -7001,7 +7035,7 @@
       </c>
       <c r="D37" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E37" s="26" t="n">
@@ -7047,7 +7081,7 @@
       </c>
       <c r="D38" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E38" s="26" t="n">
@@ -7093,7 +7127,7 @@
       </c>
       <c r="D39" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E39" s="26" t="n">
@@ -7134,12 +7168,12 @@
       </c>
       <c r="C40" s="25" t="inlineStr">
         <is>
-          <t>Autonomía aproximada reportada (horas/minutos)</t>
+          <t>¿Cuánto dura la batería aproximadamente?</t>
         </is>
       </c>
       <c r="D40" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>AUTON</t>
         </is>
       </c>
       <c r="E40" s="26" t="n">
@@ -7231,7 +7265,7 @@
       </c>
       <c r="D42" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E42" s="26" t="n">
@@ -7277,7 +7311,7 @@
       </c>
       <c r="D43" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E43" s="26" t="n">
@@ -7318,12 +7352,12 @@
       </c>
       <c r="C44" s="25" t="inlineStr">
         <is>
-          <t>¿En qué zona se calienta (batería, cámara, parte superior)?</t>
+          <t>¿En qué zona se calienta?</t>
         </is>
       </c>
       <c r="D44" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>ZONAC</t>
         </is>
       </c>
       <c r="E44" s="26" t="n">
@@ -7369,7 +7403,7 @@
       </c>
       <c r="D45" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E45" s="26" t="n">
@@ -7415,7 +7449,7 @@
       </c>
       <c r="D46" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E46" s="26" t="n">
@@ -7461,7 +7495,7 @@
       </c>
       <c r="D47" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E47" s="26" t="n">
@@ -7507,7 +7541,7 @@
       </c>
       <c r="D48" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>MANT</t>
         </is>
       </c>
       <c r="E48" s="26" t="n">
@@ -7553,7 +7587,7 @@
       </c>
       <c r="D49" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E49" s="26" t="n">
@@ -7599,7 +7633,7 @@
       </c>
       <c r="D50" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E50" s="26" t="n">
@@ -7737,7 +7771,7 @@
       </c>
       <c r="D53" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E53" s="26" t="n">
@@ -7783,7 +7817,7 @@
       </c>
       <c r="D54" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E54" s="26" t="n">
@@ -7829,7 +7863,7 @@
       </c>
       <c r="D55" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E55" s="26" t="n">
@@ -7875,7 +7909,7 @@
       </c>
       <c r="D56" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E56" s="26" t="n">
@@ -7921,7 +7955,7 @@
       </c>
       <c r="D57" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E57" s="26" t="n">
@@ -7967,7 +8001,7 @@
       </c>
       <c r="D58" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E58" s="26" t="n">
@@ -8105,7 +8139,7 @@
       </c>
       <c r="D61" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E61" s="26" t="n">
@@ -8151,7 +8185,7 @@
       </c>
       <c r="D62" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E62" s="26" t="n">
@@ -8197,7 +8231,7 @@
       </c>
       <c r="D63" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E63" s="26" t="n">
@@ -8243,7 +8277,7 @@
       </c>
       <c r="D64" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E64" s="26" t="n">
@@ -8289,7 +8323,7 @@
       </c>
       <c r="D65" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E65" s="26" t="n">
@@ -8335,7 +8369,7 @@
       </c>
       <c r="D66" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E66" s="26" t="n">
@@ -8381,7 +8415,7 @@
       </c>
       <c r="D67" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>ABCE</t>
         </is>
       </c>
       <c r="E67" s="26" t="n">
@@ -8427,7 +8461,7 @@
       </c>
       <c r="D68" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E68" s="26" t="n">
@@ -8468,12 +8502,12 @@
       </c>
       <c r="C69" s="25" t="inlineStr">
         <is>
-          <t>Zona donde recibió el impacto</t>
+          <t>¿En qué zona recibió el impacto?</t>
         </is>
       </c>
       <c r="D69" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>ZONAI</t>
         </is>
       </c>
       <c r="E69" s="26" t="n">
@@ -8519,7 +8553,7 @@
       </c>
       <c r="D70" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E70" s="26" t="n">
@@ -8565,7 +8599,7 @@
       </c>
       <c r="D71" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E71" s="26" t="n">
@@ -8611,7 +8645,7 @@
       </c>
       <c r="D72" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E72" s="26" t="n">
@@ -8657,7 +8691,7 @@
       </c>
       <c r="D73" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E73" s="26" t="n">
@@ -8703,7 +8737,7 @@
       </c>
       <c r="D74" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E74" s="26" t="n">
@@ -8749,7 +8783,7 @@
       </c>
       <c r="D75" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E75" s="26" t="n">
@@ -8795,7 +8829,7 @@
       </c>
       <c r="D76" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E76" s="26" t="n">
@@ -8841,7 +8875,7 @@
       </c>
       <c r="D77" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E77" s="26" t="n">
@@ -8887,7 +8921,7 @@
       </c>
       <c r="D78" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E78" s="26" t="n">
@@ -8933,7 +8967,7 @@
       </c>
       <c r="D79" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E79" s="26" t="n">
@@ -8979,7 +9013,7 @@
       </c>
       <c r="D80" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E80" s="26" t="n">
@@ -9025,7 +9059,7 @@
       </c>
       <c r="D81" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E81" s="26" t="n">
@@ -9071,7 +9105,7 @@
       </c>
       <c r="D82" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E82" s="26" t="n">
@@ -9117,7 +9151,7 @@
       </c>
       <c r="D83" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E83" s="26" t="n">
@@ -9163,7 +9197,7 @@
       </c>
       <c r="D84" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E84" s="26" t="n">
@@ -9209,7 +9243,7 @@
       </c>
       <c r="D85" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E85" s="26" t="n">
@@ -9255,7 +9289,7 @@
       </c>
       <c r="D86" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E86" s="26" t="n">
@@ -9296,12 +9330,12 @@
       </c>
       <c r="C87" s="25" t="inlineStr">
         <is>
-          <t>¿Cuándo comenzó la lentitud o el problema?</t>
+          <t>¿Desde cuándo comenzó la lentitud o el problema?</t>
         </is>
       </c>
       <c r="D87" s="24" t="inlineStr">
         <is>
-          <t>CUANDO</t>
+          <t>DESDE</t>
         </is>
       </c>
       <c r="E87" s="26" t="n">
@@ -9347,7 +9381,7 @@
       </c>
       <c r="D88" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E88" s="26" t="n">
@@ -9393,7 +9427,7 @@
       </c>
       <c r="D89" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E89" s="26" t="n">
@@ -9439,7 +9473,7 @@
       </c>
       <c r="D90" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E90" s="26" t="n">
@@ -9485,7 +9519,7 @@
       </c>
       <c r="D91" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E91" s="26" t="n">
@@ -9531,7 +9565,7 @@
       </c>
       <c r="D92" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E92" s="26" t="n">
@@ -9572,12 +9606,12 @@
       </c>
       <c r="C93" s="25" t="inlineStr">
         <is>
-          <t>¿Qué código de error aparece en la consola?</t>
+          <t>¿Qué tipo de error aparece en la consola?</t>
         </is>
       </c>
       <c r="D93" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>ERR</t>
         </is>
       </c>
       <c r="E93" s="26" t="n">
@@ -9618,12 +9652,12 @@
       </c>
       <c r="C94" s="25" t="inlineStr">
         <is>
-          <t>¿Qué programa, app o juego falla en específico?</t>
+          <t>¿Qué programa, app o juego falla?</t>
         </is>
       </c>
       <c r="D94" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>PROG</t>
         </is>
       </c>
       <c r="E94" s="26" t="n">
@@ -9669,7 +9703,7 @@
       </c>
       <c r="D95" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E95" s="26" t="n">
@@ -9715,7 +9749,7 @@
       </c>
       <c r="D96" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E96" s="26" t="n">
@@ -9761,7 +9795,7 @@
       </c>
       <c r="D97" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E97" s="26" t="n">
@@ -9807,7 +9841,7 @@
       </c>
       <c r="D98" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E98" s="26" t="n">
@@ -9853,7 +9887,7 @@
       </c>
       <c r="D99" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E99" s="26" t="n">
@@ -9894,12 +9928,12 @@
       </c>
       <c r="C100" s="25" t="inlineStr">
         <is>
-          <t>¿Qué sistema operativo y versión utiliza?</t>
+          <t>¿Qué sistema operativo utiliza?</t>
         </is>
       </c>
       <c r="D100" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="E100" s="26" t="n">
@@ -9945,7 +9979,7 @@
       </c>
       <c r="D101" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E101" s="26" t="n">
@@ -9991,7 +10025,7 @@
       </c>
       <c r="D102" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E102" s="26" t="n">
@@ -10037,7 +10071,7 @@
       </c>
       <c r="D103" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E103" s="26" t="n">
@@ -10083,7 +10117,7 @@
       </c>
       <c r="D104" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E104" s="26" t="n">
@@ -10129,7 +10163,7 @@
       </c>
       <c r="D105" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E105" s="26" t="n">
@@ -10175,7 +10209,7 @@
       </c>
       <c r="D106" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E106" s="26" t="n">
@@ -10313,7 +10347,7 @@
       </c>
       <c r="D109" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E109" s="26" t="n">
@@ -10359,7 +10393,7 @@
       </c>
       <c r="D110" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E110" s="26" t="n">
@@ -10405,7 +10439,7 @@
       </c>
       <c r="D111" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E111" s="26" t="n">
@@ -10451,7 +10485,7 @@
       </c>
       <c r="D112" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E112" s="26" t="n">
@@ -10497,7 +10531,7 @@
       </c>
       <c r="D113" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E113" s="26" t="n">
@@ -10543,7 +10577,7 @@
       </c>
       <c r="D114" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E114" s="26" t="n">
@@ -10589,7 +10623,7 @@
       </c>
       <c r="D115" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E115" s="26" t="n">
@@ -10635,7 +10669,7 @@
       </c>
       <c r="D116" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E116" s="26" t="n">
@@ -10681,7 +10715,7 @@
       </c>
       <c r="D117" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E117" s="26" t="n">
@@ -10727,7 +10761,7 @@
       </c>
       <c r="D118" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E118" s="26" t="n">
@@ -10773,7 +10807,7 @@
       </c>
       <c r="D119" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E119" s="26" t="n">
@@ -10819,7 +10853,7 @@
       </c>
       <c r="D120" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E120" s="26" t="n">
@@ -10865,7 +10899,7 @@
       </c>
       <c r="D121" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E121" s="26" t="n">
@@ -10911,7 +10945,7 @@
       </c>
       <c r="D122" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E122" s="26" t="n">
@@ -10957,7 +10991,7 @@
       </c>
       <c r="D123" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E123" s="26" t="n">
@@ -11003,7 +11037,7 @@
       </c>
       <c r="D124" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E124" s="26" t="n">
@@ -11049,7 +11083,7 @@
       </c>
       <c r="D125" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="E125" s="26" t="n">
@@ -11095,7 +11129,7 @@
       </c>
       <c r="D126" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E126" s="26" t="n">
@@ -11141,7 +11175,7 @@
       </c>
       <c r="D127" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E127" s="26" t="n">
@@ -11187,7 +11221,7 @@
       </c>
       <c r="D128" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E128" s="26" t="n">
@@ -11233,7 +11267,7 @@
       </c>
       <c r="D129" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E129" s="26" t="n">
@@ -11279,7 +11313,7 @@
       </c>
       <c r="D130" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E130" s="26" t="n">
@@ -11325,7 +11359,7 @@
       </c>
       <c r="D131" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E131" s="26" t="n">
@@ -11371,7 +11405,7 @@
       </c>
       <c r="D132" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E132" s="26" t="n">
@@ -11417,7 +11451,7 @@
       </c>
       <c r="D133" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E133" s="26" t="n">
@@ -11463,7 +11497,7 @@
       </c>
       <c r="D134" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E134" s="26" t="n">
@@ -11509,7 +11543,7 @@
       </c>
       <c r="D135" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E135" s="26" t="n">
@@ -11555,7 +11589,7 @@
       </c>
       <c r="D136" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E136" s="26" t="n">
@@ -11601,7 +11635,7 @@
       </c>
       <c r="D137" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E137" s="26" t="n">
@@ -11642,12 +11676,12 @@
       </c>
       <c r="C138" s="25" t="inlineStr">
         <is>
-          <t>¿Falla con todos los juegos o con uno solo? (indique cuál)</t>
+          <t>¿Falla con todos los discos o solo con algunos?</t>
         </is>
       </c>
       <c r="D138" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>JUE</t>
         </is>
       </c>
       <c r="E138" s="26" t="n">
@@ -11693,7 +11727,7 @@
       </c>
       <c r="D139" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E139" s="26" t="n">
@@ -11739,7 +11773,7 @@
       </c>
       <c r="D140" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E140" s="26" t="n">
@@ -11785,7 +11819,7 @@
       </c>
       <c r="D141" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E141" s="26" t="n">
@@ -11831,7 +11865,7 @@
       </c>
       <c r="D142" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E142" s="26" t="n">
@@ -11877,7 +11911,7 @@
       </c>
       <c r="D143" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E143" s="26" t="n">
@@ -11923,7 +11957,7 @@
       </c>
       <c r="D144" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E144" s="26" t="n">
@@ -11969,7 +12003,7 @@
       </c>
       <c r="D145" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>NCTRL</t>
         </is>
       </c>
       <c r="E145" s="26" t="n">
@@ -12015,7 +12049,7 @@
       </c>
       <c r="D146" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E146" s="26" t="n">
@@ -12061,7 +12095,7 @@
       </c>
       <c r="D147" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E147" s="26" t="n">
@@ -12107,7 +12141,7 @@
       </c>
       <c r="D148" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E148" s="26" t="n">
@@ -12153,7 +12187,7 @@
       </c>
       <c r="D149" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E149" s="26" t="n">
@@ -12199,7 +12233,7 @@
       </c>
       <c r="D150" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>YNS</t>
         </is>
       </c>
       <c r="E150" s="26" t="n">
@@ -12240,12 +12274,12 @@
       </c>
       <c r="C151" s="25" t="inlineStr">
         <is>
-          <t>Describa la otra falla o condición</t>
+          <t>¿Cuál es la otra falla o condición?</t>
         </is>
       </c>
       <c r="D151" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>OTRAF</t>
         </is>
       </c>
       <c r="E151" s="26" t="n">
@@ -12286,12 +12320,12 @@
       </c>
       <c r="C152" s="25" t="inlineStr">
         <is>
-          <t>¿Qué soluciones ya intentó el cliente?</t>
+          <t>¿Qué solución ya intentó el cliente?</t>
         </is>
       </c>
       <c r="D152" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="E152" s="26" t="n">
@@ -12834,12 +12868,12 @@
       </c>
       <c r="C164" s="25" t="inlineStr">
         <is>
-          <t>Otro daño visible (describa)</t>
+          <t>¿Qué otro daño visible tiene?</t>
         </is>
       </c>
       <c r="D164" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>DANO</t>
         </is>
       </c>
       <c r="E164" s="26" t="n">
@@ -12885,7 +12919,7 @@
       </c>
       <c r="D165" s="24" t="inlineStr">
         <is>
-          <t>YNS</t>
+          <t>YNC</t>
         </is>
       </c>
       <c r="E165" s="26" t="n">
@@ -12931,7 +12965,7 @@
       </c>
       <c r="D166" s="24" t="inlineStr">
         <is>
-          <t>YNS</t>
+          <t>YNC</t>
         </is>
       </c>
       <c r="E166" s="26" t="n">
@@ -12977,7 +13011,7 @@
       </c>
       <c r="D167" s="24" t="inlineStr">
         <is>
-          <t>YNS</t>
+          <t>YNC</t>
         </is>
       </c>
       <c r="E167" s="26" t="n">
@@ -13023,7 +13057,7 @@
       </c>
       <c r="D168" s="24" t="inlineStr">
         <is>
-          <t>YNS</t>
+          <t>YNC</t>
         </is>
       </c>
       <c r="E168" s="26" t="n">
@@ -13938,12 +13972,12 @@
       </c>
       <c r="C188" s="25" t="inlineStr">
         <is>
-          <t>¿Entregó otro accesorio? (descríbalo)</t>
+          <t>¿Entregó otro accesorio?</t>
         </is>
       </c>
       <c r="D188" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>YN</t>
         </is>
       </c>
       <c r="E188" s="26" t="n">
@@ -14265,7 +14299,7 @@
       </c>
       <c r="D195" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E195" s="26" t="n">
@@ -14311,7 +14345,7 @@
       </c>
       <c r="D196" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E196" s="26" t="n">
@@ -14357,7 +14391,7 @@
       </c>
       <c r="D197" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E197" s="26" t="n">
@@ -14403,7 +14437,7 @@
       </c>
       <c r="D198" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E198" s="26" t="n">
@@ -14449,7 +14483,7 @@
       </c>
       <c r="D199" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E199" s="26" t="n">
@@ -14495,7 +14529,7 @@
       </c>
       <c r="D200" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E200" s="26" t="n">
@@ -14541,7 +14575,7 @@
       </c>
       <c r="D201" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E201" s="26" t="n">
@@ -14587,7 +14621,7 @@
       </c>
       <c r="D202" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E202" s="26" t="n">
@@ -14633,7 +14667,7 @@
       </c>
       <c r="D203" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E203" s="26" t="n">
@@ -14679,7 +14713,7 @@
       </c>
       <c r="D204" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E204" s="26" t="n">
@@ -14725,7 +14759,7 @@
       </c>
       <c r="D205" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E205" s="26" t="n">
@@ -14771,7 +14805,7 @@
       </c>
       <c r="D206" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E206" s="26" t="n">
@@ -14817,7 +14851,7 @@
       </c>
       <c r="D207" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E207" s="26" t="n">
@@ -14863,7 +14897,7 @@
       </c>
       <c r="D208" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E208" s="26" t="n">
@@ -14909,7 +14943,7 @@
       </c>
       <c r="D209" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E209" s="26" t="n">
@@ -14955,7 +14989,7 @@
       </c>
       <c r="D210" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E210" s="26" t="n">
@@ -15001,7 +15035,7 @@
       </c>
       <c r="D211" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E211" s="26" t="n">
@@ -15047,7 +15081,7 @@
       </c>
       <c r="D212" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E212" s="26" t="n">
@@ -15093,7 +15127,7 @@
       </c>
       <c r="D213" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E213" s="26" t="n">
@@ -15139,7 +15173,7 @@
       </c>
       <c r="D214" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E214" s="26" t="n">
@@ -15185,7 +15219,7 @@
       </c>
       <c r="D215" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E215" s="26" t="n">
@@ -15231,7 +15265,7 @@
       </c>
       <c r="D216" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E216" s="26" t="n">
@@ -15277,7 +15311,7 @@
       </c>
       <c r="D217" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E217" s="26" t="n">
@@ -15323,7 +15357,7 @@
       </c>
       <c r="D218" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E218" s="26" t="n">
@@ -15369,7 +15403,7 @@
       </c>
       <c r="D219" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E219" s="26" t="n">
@@ -15415,7 +15449,7 @@
       </c>
       <c r="D220" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E220" s="26" t="n">
@@ -15461,7 +15495,7 @@
       </c>
       <c r="D221" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E221" s="26" t="n">
@@ -15507,7 +15541,7 @@
       </c>
       <c r="D222" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E222" s="26" t="n">
@@ -15553,7 +15587,7 @@
       </c>
       <c r="D223" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E223" s="26" t="n">
@@ -15599,7 +15633,7 @@
       </c>
       <c r="D224" s="24" t="inlineStr">
         <is>
-          <t>YN</t>
+          <t>FUN</t>
         </is>
       </c>
       <c r="E224" s="26" t="n">
@@ -15866,7 +15900,7 @@
       </c>
       <c r="C230" s="25" t="inlineStr">
         <is>
-          <t>Contraseña / PIN requerido para pruebas</t>
+          <t>¿Cómo se maneja la contraseña / PIN para las pruebas?</t>
         </is>
       </c>
       <c r="D230" s="24" t="inlineStr">
@@ -15912,12 +15946,12 @@
       </c>
       <c r="C231" s="25" t="inlineStr">
         <is>
-          <t>Nombre del cliente que autoriza</t>
+          <t>¿El cliente firmó la orden de recepción?</t>
         </is>
       </c>
       <c r="D231" s="24" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>YN</t>
         </is>
       </c>
       <c r="E231" s="26" t="n">
@@ -15958,7 +15992,7 @@
       </c>
       <c r="C232" s="25" t="inlineStr">
         <is>
-          <t>Nombre de quien recibe por RCP</t>
+          <t>Contraseña / PIN (escríbalo solo si el cliente lo proporciona)</t>
         </is>
       </c>
       <c r="D232" s="24" t="inlineStr">
@@ -19750,7 +19784,7 @@
       <formula1>"1,0"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"YN,YNS,TXT,CUANDO,MOM,LIQ,E_PANT,E_CARC,PIN,HEAD"</formula1>
+      <formula1>"YN,YNS,YNC,FUN,TXT,HEAD"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19763,7 +19797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y15"/>
+  <dimension ref="A1:AU15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -19782,6 +19816,28 @@
     <col width="24" customWidth="1" min="23" max="23"/>
     <col width="24" customWidth="1" min="24" max="24"/>
     <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="24" customWidth="1" min="26" max="26"/>
+    <col width="24" customWidth="1" min="27" max="27"/>
+    <col width="24" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="24" customWidth="1" min="30" max="30"/>
+    <col width="24" customWidth="1" min="31" max="31"/>
+    <col width="24" customWidth="1" min="32" max="32"/>
+    <col width="24" customWidth="1" min="33" max="33"/>
+    <col width="24" customWidth="1" min="34" max="34"/>
+    <col width="24" customWidth="1" min="35" max="35"/>
+    <col width="24" customWidth="1" min="36" max="36"/>
+    <col width="24" customWidth="1" min="37" max="37"/>
+    <col width="24" customWidth="1" min="38" max="38"/>
+    <col width="24" customWidth="1" min="39" max="39"/>
+    <col width="24" customWidth="1" min="40" max="40"/>
+    <col width="24" customWidth="1" min="41" max="41"/>
+    <col width="24" customWidth="1" min="42" max="42"/>
+    <col width="24" customWidth="1" min="43" max="43"/>
+    <col width="24" customWidth="1" min="44" max="44"/>
+    <col width="24" customWidth="1" min="45" max="45"/>
+    <col width="24" customWidth="1" min="46" max="46"/>
+    <col width="24" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19827,30 +19883,140 @@
       </c>
       <c r="T1" s="28" t="inlineStr">
         <is>
+          <t>L_YNC</t>
+        </is>
+      </c>
+      <c r="U1" s="28" t="inlineStr">
+        <is>
+          <t>L_FUN</t>
+        </is>
+      </c>
+      <c r="V1" s="28" t="inlineStr">
+        <is>
+          <t>L_FALLAP</t>
+        </is>
+      </c>
+      <c r="W1" s="28" t="inlineStr">
+        <is>
+          <t>L_DESDE</t>
+        </is>
+      </c>
+      <c r="X1" s="28" t="inlineStr">
+        <is>
+          <t>L_PERM</t>
+        </is>
+      </c>
+      <c r="Y1" s="28" t="inlineStr">
+        <is>
+          <t>L_ENC</t>
+        </is>
+      </c>
+      <c r="Z1" s="28" t="inlineStr">
+        <is>
+          <t>L_OTRAF</t>
+        </is>
+      </c>
+      <c r="AA1" s="28" t="inlineStr">
+        <is>
+          <t>L_LUZ</t>
+        </is>
+      </c>
+      <c r="AB1" s="28" t="inlineStr">
+        <is>
+          <t>L_SENAL</t>
+        </is>
+      </c>
+      <c r="AC1" s="28" t="inlineStr">
+        <is>
+          <t>L_AUTON</t>
+        </is>
+      </c>
+      <c r="AD1" s="28" t="inlineStr">
+        <is>
+          <t>L_ZONAC</t>
+        </is>
+      </c>
+      <c r="AE1" s="28" t="inlineStr">
+        <is>
+          <t>L_MANT</t>
+        </is>
+      </c>
+      <c r="AF1" s="28" t="inlineStr">
+        <is>
+          <t>L_ABCE</t>
+        </is>
+      </c>
+      <c r="AG1" s="28" t="inlineStr">
+        <is>
+          <t>L_ZONAI</t>
+        </is>
+      </c>
+      <c r="AH1" s="28" t="inlineStr">
+        <is>
+          <t>L_ERR</t>
+        </is>
+      </c>
+      <c r="AI1" s="28" t="inlineStr">
+        <is>
+          <t>L_PROG</t>
+        </is>
+      </c>
+      <c r="AJ1" s="28" t="inlineStr">
+        <is>
+          <t>L_SO</t>
+        </is>
+      </c>
+      <c r="AK1" s="28" t="inlineStr">
+        <is>
+          <t>L_TEL</t>
+        </is>
+      </c>
+      <c r="AL1" s="28" t="inlineStr">
+        <is>
+          <t>L_JUE</t>
+        </is>
+      </c>
+      <c r="AM1" s="28" t="inlineStr">
+        <is>
+          <t>L_NCTRL</t>
+        </is>
+      </c>
+      <c r="AN1" s="28" t="inlineStr">
+        <is>
+          <t>L_SOL</t>
+        </is>
+      </c>
+      <c r="AO1" s="28" t="inlineStr">
+        <is>
+          <t>L_DANO</t>
+        </is>
+      </c>
+      <c r="AP1" s="28" t="inlineStr">
+        <is>
           <t>L_CUANDO</t>
         </is>
       </c>
-      <c r="U1" s="28" t="inlineStr">
+      <c r="AQ1" s="28" t="inlineStr">
         <is>
           <t>L_MOM</t>
         </is>
       </c>
-      <c r="V1" s="28" t="inlineStr">
+      <c r="AR1" s="28" t="inlineStr">
         <is>
           <t>L_LIQ</t>
         </is>
       </c>
-      <c r="W1" s="28" t="inlineStr">
+      <c r="AS1" s="28" t="inlineStr">
         <is>
           <t>L_E_PANT</t>
         </is>
       </c>
-      <c r="X1" s="28" t="inlineStr">
+      <c r="AT1" s="28" t="inlineStr">
         <is>
           <t>L_E_CARC</t>
         </is>
       </c>
-      <c r="Y1" s="28" t="inlineStr">
+      <c r="AU1" s="28" t="inlineStr">
         <is>
           <t>L_PIN</t>
         </is>
@@ -19899,32 +20065,142 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Funciona</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>No enciende</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
           <t>Hoy</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Permanente</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Menos de 30 minutos</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Parte trasera</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Nunca</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Abierta</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Pantalla</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>No aparece error</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>Todos por igual</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Windows 11</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>iPhone</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>Todos los discos</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>Hoy</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>Uso normal</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>Agua</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>Sin daño</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AT2" t="inlineStr">
         <is>
           <t>Buen estado</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Proporcionado</t>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>Proporcionó la contraseña</t>
         </is>
       </c>
     </row>
@@ -19971,32 +20247,142 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>No funciona</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>No carga / batería</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Últimos 3 días</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Sucede algunas veces</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Pantalla</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Roja</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Luz</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>30 min a 1 hora</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Parte superior</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Menos de 6 meses</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Cerrada</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Esquina</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Error de actualización</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>Navegador</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Windows 10</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>Solo algunos</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>Reinició el equipo</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>Rayones leves</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
           <t>Esta semana</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="AQ3" t="inlineStr">
         <is>
           <t>Juegos</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="AR3" t="inlineStr">
         <is>
           <t>Agua de piscina</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="AS3" t="inlineStr">
         <is>
           <t>Rayones</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="AT3" t="inlineStr">
         <is>
           <t>Rayones</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Cliente lo ingresará</t>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>Cliente la ingresará en la prueba</t>
         </is>
       </c>
     </row>
@@ -20038,32 +20424,142 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
+          <t>No fue posible comprobar</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>No probado</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Pantalla dañada o sin imagen</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Esta semana</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>No sabe</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Intermitente</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Batería o carga</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Vibración</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>1 a 3 horas</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Cerca de la batería</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>6 a 12 meses</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>No sabe</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Parte trasera</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Error de disco</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Juegos</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Windows 7 o anterior</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>No sabe</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Un solo disco</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Cambió cargador o cable</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Golpes</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
           <t>Este mes</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="AQ4" t="inlineStr">
         <is>
           <t>Cargando</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="AR4" t="inlineStr">
         <is>
           <t>Agua de mar</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="AS4" t="inlineStr">
         <is>
           <t>Quebrada</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="AT4" t="inlineStr">
         <is>
           <t>Golpes o abolladuras</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>No proporcionado</t>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>No proporcionó contraseña</t>
         </is>
       </c>
     </row>
@@ -20098,32 +20594,117 @@
           <t>Contacto con líquido</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Se calienta o se apaga</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Este mes</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>No sé</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Sonido</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Blanca</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Sonido</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>3 a 6 horas</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Cerca de la cámara</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Más de 1 año</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>Lateral</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>Error de red</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>Programas de trabajo</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>macOS</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>3 o más</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Restableció de fábrica</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>Grietas</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
         <is>
           <t>Hace más de 1 mes</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="AQ5" t="inlineStr">
         <is>
           <t>Siempre</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="AR5" t="inlineStr">
         <is>
           <t>Café</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="AS5" t="inlineStr">
         <is>
           <t>Manchas o líneas</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="AT5" t="inlineStr">
         <is>
           <t>Carcasa rota</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AU5" t="inlineStr">
         <is>
           <t>No aplica</t>
         </is>
@@ -20150,12 +20731,82 @@
           <t>Golpe / Caída</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Lentitud o se congela</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Hace 1 a 3 meses</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Naranja</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Varias señales</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>Más de 6 horas</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
         <is>
           <t>No sabe</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>Parte inferior</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>Error de hardware</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Redes sociales / mensajería</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>Linux</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Lo llevó a otro taller</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>Piezas sueltas</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>No sabe</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
         <is>
           <t>Gaseosa</t>
         </is>
@@ -20184,6 +20835,66 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
+          <t>Golpe o caída</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Hace más de 3 meses</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Señal / Wi-Fi</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>No sabe</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>No sabe</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>Parte superior</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>No sabe</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>Ninguno en específico</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>No sabe</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>Lo intentó reparar personalmente</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>Faltan piezas</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
           <t>Alcohol</t>
         </is>
       </c>
@@ -20211,6 +20922,46 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
+          <t>Contacto con líquido</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>No sabe</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Botones</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Parpadea</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>Varias zonas</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>Otro (ver Detalle)</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>Otra (ver Detalle)</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>Otro (ver Detalle)</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
           <t>Otro líquido</t>
         </is>
       </c>
@@ -20236,6 +20987,21 @@
           <t>Disco / Almacenamiento</t>
         </is>
       </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Sin sonido / cámara / micrófono</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Lentitud</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>No sabe</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="F10" s="29" t="inlineStr">
@@ -20258,6 +21024,16 @@
           <t>Cuenta / Bloqueo</t>
         </is>
       </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Sin señal o conexión</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Otra (ver Detalle)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="F11" s="29" t="inlineStr">
@@ -20280,6 +21056,11 @@
           <t>Audio / Cámara / Micrófono</t>
         </is>
       </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Botones o teclado</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="F12" s="29" t="inlineStr">
@@ -20300,6 +21081,11 @@
       <c r="I12" s="29" t="inlineStr">
         <is>
           <t>Red / Señal / Conectividad</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Otra falla</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reordena la hoja de recepción: alertas al lado de los datos, tabla justo debajo y columnas alineadas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vbz2Sf1pkMwtP6vBTAs1UZ
</commit_message>
<xml_diff>
--- a/RCP_Checklist_Recepcion_Tecnica.xlsx
+++ b/RCP_Checklist_Recepcion_Tecnica.xlsx
@@ -54,7 +54,7 @@
     <definedName name="L_YN">Listas!$AY$2:$AY$3</definedName>
     <definedName name="L_YNS">Listas!$AZ$2:$AZ$4</definedName>
     <definedName name="L_TXT">Listas!$BA$2:$BA$2</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Recepción'!$21:$21</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Recepción'!$16:$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preguntas'!$A$1:$F$775</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -127,14 +127,14 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="002E75B6"/>
-      <sz val="10"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="009C0006"/>
+      <i val="1"/>
+      <color rgb="002E75B6"/>
       <sz val="10"/>
     </font>
     <font>
@@ -144,7 +144,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -173,12 +173,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF8DC"/>
         <bgColor rgb="00FFF8DC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -234,22 +228,20 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -261,7 +253,7 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -850,21 +842,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:L121"/>
+  <dimension ref="B1:M116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="64" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
     <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
     <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
     <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -887,6 +880,11 @@
           <t>DATOS DEL EQUIPO Y DEL CLIENTE</t>
         </is>
       </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>ALERTAS AUTOMÁTICAS</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="21" customHeight="1">
       <c r="B5" s="7" t="inlineStr">
@@ -897,6 +895,15 @@
       <c r="C5" s="8" t="n"/>
       <c r="D5" s="9" t="n"/>
       <c r="E5" s="10" t="n"/>
+      <c r="F5" s="11">
+        <f>IF($D$5="","",IF(M5&amp;M6&amp;M7&amp;M8&amp;M9="","Sin alertas por ahora.",M5&amp;M6&amp;M7&amp;M8&amp;M9))</f>
+        <v/>
+      </c>
+      <c r="G5" s="12" t="n"/>
+      <c r="M5">
+        <f>IF(COUNTIFS($D$17:$D$116,"¿Ha tenido contacto con agua, humedad o algún líquido?",$E$17:$E$116,"Sí")&gt;0,"• ALTA PRIORIDAD · Ingresa por CONTAMINACIÓN DE LÍQUIDO: registrarlo en la orden; no encender ni conectar al cargador."&amp;CHAR(10),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="21" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
@@ -907,6 +914,12 @@
       <c r="C6" s="8" t="n"/>
       <c r="D6" s="9" t="n"/>
       <c r="E6" s="10" t="n"/>
+      <c r="F6" s="12" t="n"/>
+      <c r="G6" s="12" t="n"/>
+      <c r="M6">
+        <f>IF(SUMPRODUCT(ISNUMBER(SEARCH("inflada",$D$17:$D$116))*($E$17:$E$116="Sí"))&gt;0,"• ALTA PRIORIDAD · Batería inflada / equipo deformado: riesgo de seguridad, manipular con cuidado y aislar el equipo."&amp;CHAR(10),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="21" customHeight="1">
       <c r="B7" s="7" t="inlineStr">
@@ -917,6 +930,12 @@
       <c r="C7" s="8" t="n"/>
       <c r="D7" s="9" t="n"/>
       <c r="E7" s="10" t="n"/>
+      <c r="F7" s="12" t="n"/>
+      <c r="G7" s="12" t="n"/>
+      <c r="M7">
+        <f>IF(AND(COUNTIFS($D$17:$D$116,"¿Tiene información importante que no puede perder?",$E$17:$E$116,"Sí")&gt;0,COUNTIFS($D$17:$D$116,"¿Tiene respaldo reciente de su información?",$E$17:$E$116,"Sí")=0),"• DATOS EN RIESGO · Información importante SIN respaldo confirmado: reforzar la autorización antes de intervenir."&amp;CHAR(10),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="21" customHeight="1">
       <c r="B8" s="7" t="inlineStr">
@@ -927,6 +946,12 @@
       <c r="C8" s="8" t="n"/>
       <c r="D8" s="9" t="n"/>
       <c r="E8" s="10" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="M8">
+        <f>IF(COUNTIFS($D$17:$D$116,"¿Ha sido abierto o reparado anteriormente?",$E$17:$E$116,"Sí")&gt;0,"• Equipo abierto o reparado antes: fotografiar señales de apertura y anotar quién lo intervino."&amp;CHAR(10),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="21" customHeight="1">
       <c r="B9" s="7" t="inlineStr">
@@ -937,6 +962,12 @@
       <c r="C9" s="8" t="n"/>
       <c r="D9" s="9" t="n"/>
       <c r="E9" s="10" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="M9">
+        <f>IF(COUNTIFS($D$17:$D$116,"¿Sufrió algún golpe o caída recientemente?",$E$17:$E$116,"Sí")&gt;0,"• Golpe o caída reportado: documentar la zona del impacto y fotografiar daños existentes."&amp;CHAR(10),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="21" customHeight="1">
       <c r="B10" s="7" t="inlineStr">
@@ -947,6 +978,8 @@
       <c r="C10" s="8" t="n"/>
       <c r="D10" s="9" t="n"/>
       <c r="E10" s="10" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="12" t="n"/>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="B11" s="7" t="inlineStr">
@@ -957,6 +990,8 @@
       <c r="C11" s="8" t="n"/>
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="10" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="B12" s="7" t="inlineStr">
@@ -965,88 +1000,211 @@
         </is>
       </c>
       <c r="C12" s="8" t="n"/>
-      <c r="D12" s="11" t="n"/>
+      <c r="D12" s="13" t="n"/>
       <c r="E12" s="10" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+    </row>
+    <row r="13" ht="21" customHeight="1">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Nivel de atención</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="14">
+        <f>IF(D5="","",IF(OR(COUNTIFS($D$17:$D$116,"¿Ha tenido contacto con agua, humedad o algún líquido?",$E$17:$E$116,"Sí")&gt;0,SUMPRODUCT(ISNUMBER(SEARCH("inflada",$D$17:$D$116))*($E$17:$E$116="Sí"))&gt;0),"ALTA PRIORIDAD","Normal"))</f>
+        <v/>
+      </c>
+      <c r="E13" s="12" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Nivel de atención</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="12">
-        <f>IF(D5="","",IF(OR(COUNTIFS($D$22:$D$121,"¿Ha tenido contacto con agua, humedad o algún líquido?",$E$22:$E$121,"Sí")&gt;0,SUMPRODUCT(ISNUMBER(SEARCH("inflada",$D$22:$D$121))*($E$22:$E$121="Sí"))&gt;0),"ALTA PRIORIDAD","Normal"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="13">
-        <f>IF(D5="","Paso 1: elija el tipo de equipo.","Preguntas respondidas: "&amp;COUNTA(E22:E121)&amp;" de "&amp;COUNTA(D22:D121))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="14" customHeight="1">
-      <c r="B16" s="14">
-        <f>IF(COUNTIFS($D$22:$D$121,"¿Ha tenido contacto con agua, humedad o algún líquido?",$E$22:$E$121,"Sí")&gt;0,"ALTA PRIORIDAD · Ingresa por CONTAMINACIÓN DE LÍQUIDO: registrarlo en la orden; no encender ni conectar al cargador.","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="14" customHeight="1">
-      <c r="B17" s="14">
-        <f>IF(SUMPRODUCT(ISNUMBER(SEARCH("inflada",$D$22:$D$121))*($E$22:$E$121="Sí"))&gt;0,"ALTA PRIORIDAD · Batería inflada / equipo deformado: riesgo de seguridad, manipular con cuidado y aislar el equipo.","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="14" customHeight="1">
-      <c r="B18" s="14">
-        <f>IF(AND(COUNTIFS($D$22:$D$121,"¿Tiene información importante que no puede perder?",$E$22:$E$121,"Sí")&gt;0,COUNTIFS($D$22:$D$121,"¿Tiene respaldo reciente de su información?",$E$22:$E$121,"Sí")=0),"DATOS EN RIESGO · Información importante SIN respaldo confirmado: reforzar la autorización antes de intervenir.","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="14" customHeight="1">
-      <c r="B19" s="14">
-        <f>IF(COUNTIFS($D$22:$D$121,"¿Ha sido abierto o reparado anteriormente?",$E$22:$E$121,"Sí")&gt;0,"Equipo abierto o reparado antes: fotografiar señales de apertura y anotar quién lo intervino.","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="14" customHeight="1">
-      <c r="B20" s="14">
-        <f>IF(COUNTIFS($D$22:$D$121,"¿Sufrió algún golpe o caída recientemente?",$E$22:$E$121,"Sí")&gt;0,"Golpe o caída reportado: documentar la zona del impacto y fotografiar daños existentes.","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B14" s="15">
+        <f>IF(D5="","Paso 1: elija el tipo de equipo.","Preguntas respondidas: "&amp;COUNTA(E17:E116)&amp;" de "&amp;COUNTA(D17:D116))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="6" customHeight="1"/>
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>N.º</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>① Categoría / Falla</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D16" s="16" t="inlineStr">
         <is>
           <t>② Pregunta</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>③ Respuesta</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>Observación (opcional)</t>
         </is>
       </c>
-      <c r="G21" s="16" t="inlineStr"/>
-    </row>
-    <row r="22">
+      <c r="G16" s="16" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="21" customHeight="1">
+      <c r="B17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="20">
+        <f>IF(AND(D17&lt;&gt;"",I17=""),"⚠ revisar","")</f>
+        <v/>
+      </c>
+      <c r="H17">
+        <f>IF(OR($D$5="",C17=""),"",$D$5&amp;"|"&amp;C17)</f>
+        <v/>
+      </c>
+      <c r="I17">
+        <f>IF(OR(H17="",D17=""),"",IFERROR(MATCH(H17&amp;"|"&amp;D17,Preguntas!$F$2:$F$1000,0),""))</f>
+        <v/>
+      </c>
+      <c r="K17">
+        <f>IF(I17="","",INDEX(Preguntas!$D$2:$D$1000,I17))</f>
+        <v/>
+      </c>
+      <c r="L17">
+        <f>IF(K17="","L_YN","L_"&amp;K17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="B18" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="18" t="n"/>
+      <c r="D18" s="18" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="18" t="n"/>
+      <c r="G18" s="20">
+        <f>IF(AND(D18&lt;&gt;"",I18=""),"⚠ revisar","")</f>
+        <v/>
+      </c>
+      <c r="H18">
+        <f>IF(OR($D$5="",C18=""),"",$D$5&amp;"|"&amp;C18)</f>
+        <v/>
+      </c>
+      <c r="I18">
+        <f>IF(OR(H18="",D18=""),"",IFERROR(MATCH(H18&amp;"|"&amp;D18,Preguntas!$F$2:$F$1000,0),""))</f>
+        <v/>
+      </c>
+      <c r="K18">
+        <f>IF(I18="","",INDEX(Preguntas!$D$2:$D$1000,I18))</f>
+        <v/>
+      </c>
+      <c r="L18">
+        <f>IF(K18="","L_YN","L_"&amp;K18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="21" customHeight="1">
+      <c r="B19" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="20">
+        <f>IF(AND(D19&lt;&gt;"",I19=""),"⚠ revisar","")</f>
+        <v/>
+      </c>
+      <c r="H19">
+        <f>IF(OR($D$5="",C19=""),"",$D$5&amp;"|"&amp;C19)</f>
+        <v/>
+      </c>
+      <c r="I19">
+        <f>IF(OR(H19="",D19=""),"",IFERROR(MATCH(H19&amp;"|"&amp;D19,Preguntas!$F$2:$F$1000,0),""))</f>
+        <v/>
+      </c>
+      <c r="K19">
+        <f>IF(I19="","",INDEX(Preguntas!$D$2:$D$1000,I19))</f>
+        <v/>
+      </c>
+      <c r="L19">
+        <f>IF(K19="","L_YN","L_"&amp;K19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="21" customHeight="1">
+      <c r="B20" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="18" t="n"/>
+      <c r="D20" s="18" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="18" t="n"/>
+      <c r="G20" s="20">
+        <f>IF(AND(D20&lt;&gt;"",I20=""),"⚠ revisar","")</f>
+        <v/>
+      </c>
+      <c r="H20">
+        <f>IF(OR($D$5="",C20=""),"",$D$5&amp;"|"&amp;C20)</f>
+        <v/>
+      </c>
+      <c r="I20">
+        <f>IF(OR(H20="",D20=""),"",IFERROR(MATCH(H20&amp;"|"&amp;D20,Preguntas!$F$2:$F$1000,0),""))</f>
+        <v/>
+      </c>
+      <c r="K20">
+        <f>IF(I20="","",INDEX(Preguntas!$D$2:$D$1000,I20))</f>
+        <v/>
+      </c>
+      <c r="L20">
+        <f>IF(K20="","L_YN","L_"&amp;K20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="21" customHeight="1">
+      <c r="B21" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="18" t="n"/>
+      <c r="D21" s="18" t="n"/>
+      <c r="E21" s="19" t="n"/>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="20">
+        <f>IF(AND(D21&lt;&gt;"",I21=""),"⚠ revisar","")</f>
+        <v/>
+      </c>
+      <c r="H21">
+        <f>IF(OR($D$5="",C21=""),"",$D$5&amp;"|"&amp;C21)</f>
+        <v/>
+      </c>
+      <c r="I21">
+        <f>IF(OR(H21="",D21=""),"",IFERROR(MATCH(H21&amp;"|"&amp;D21,Preguntas!$F$2:$F$1000,0),""))</f>
+        <v/>
+      </c>
+      <c r="K21">
+        <f>IF(I21="","",INDEX(Preguntas!$D$2:$D$1000,I21))</f>
+        <v/>
+      </c>
+      <c r="L21">
+        <f>IF(K21="","L_YN","L_"&amp;K21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="21" customHeight="1">
       <c r="B22" s="17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C22" s="18" t="n"/>
       <c r="D22" s="18" t="n"/>
@@ -1073,9 +1231,9 @@
         <v/>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="21" customHeight="1">
       <c r="B23" s="17" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C23" s="18" t="n"/>
       <c r="D23" s="18" t="n"/>
@@ -1102,9 +1260,9 @@
         <v/>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="21" customHeight="1">
       <c r="B24" s="17" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C24" s="18" t="n"/>
       <c r="D24" s="18" t="n"/>
@@ -1131,9 +1289,9 @@
         <v/>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="21" customHeight="1">
       <c r="B25" s="17" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C25" s="18" t="n"/>
       <c r="D25" s="18" t="n"/>
@@ -1160,9 +1318,9 @@
         <v/>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="21" customHeight="1">
       <c r="B26" s="17" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C26" s="18" t="n"/>
       <c r="D26" s="18" t="n"/>
@@ -1189,9 +1347,9 @@
         <v/>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="21" customHeight="1">
       <c r="B27" s="17" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C27" s="18" t="n"/>
       <c r="D27" s="18" t="n"/>
@@ -1218,9 +1376,9 @@
         <v/>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="21" customHeight="1">
       <c r="B28" s="17" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C28" s="18" t="n"/>
       <c r="D28" s="18" t="n"/>
@@ -1247,9 +1405,9 @@
         <v/>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="21" customHeight="1">
       <c r="B29" s="17" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C29" s="18" t="n"/>
       <c r="D29" s="18" t="n"/>
@@ -1276,9 +1434,9 @@
         <v/>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="21" customHeight="1">
       <c r="B30" s="17" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C30" s="18" t="n"/>
       <c r="D30" s="18" t="n"/>
@@ -1305,9 +1463,9 @@
         <v/>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="21" customHeight="1">
       <c r="B31" s="17" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C31" s="18" t="n"/>
       <c r="D31" s="18" t="n"/>
@@ -1334,9 +1492,9 @@
         <v/>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="21" customHeight="1">
       <c r="B32" s="17" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C32" s="18" t="n"/>
       <c r="D32" s="18" t="n"/>
@@ -1363,9 +1521,9 @@
         <v/>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="21" customHeight="1">
       <c r="B33" s="17" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C33" s="18" t="n"/>
       <c r="D33" s="18" t="n"/>
@@ -1392,9 +1550,9 @@
         <v/>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="21" customHeight="1">
       <c r="B34" s="17" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C34" s="18" t="n"/>
       <c r="D34" s="18" t="n"/>
@@ -1421,9 +1579,9 @@
         <v/>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="21" customHeight="1">
       <c r="B35" s="17" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C35" s="18" t="n"/>
       <c r="D35" s="18" t="n"/>
@@ -1450,9 +1608,9 @@
         <v/>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="21" customHeight="1">
       <c r="B36" s="17" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C36" s="18" t="n"/>
       <c r="D36" s="18" t="n"/>
@@ -1479,9 +1637,9 @@
         <v/>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="21" customHeight="1">
       <c r="B37" s="17" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C37" s="18" t="n"/>
       <c r="D37" s="18" t="n"/>
@@ -1508,9 +1666,9 @@
         <v/>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="21" customHeight="1">
       <c r="B38" s="17" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C38" s="18" t="n"/>
       <c r="D38" s="18" t="n"/>
@@ -1537,9 +1695,9 @@
         <v/>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="21" customHeight="1">
       <c r="B39" s="17" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C39" s="18" t="n"/>
       <c r="D39" s="18" t="n"/>
@@ -1566,9 +1724,9 @@
         <v/>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="21" customHeight="1">
       <c r="B40" s="17" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C40" s="18" t="n"/>
       <c r="D40" s="18" t="n"/>
@@ -1595,9 +1753,9 @@
         <v/>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="21" customHeight="1">
       <c r="B41" s="17" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C41" s="18" t="n"/>
       <c r="D41" s="18" t="n"/>
@@ -1624,9 +1782,9 @@
         <v/>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="21" customHeight="1">
       <c r="B42" s="17" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C42" s="18" t="n"/>
       <c r="D42" s="18" t="n"/>
@@ -1653,9 +1811,9 @@
         <v/>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="21" customHeight="1">
       <c r="B43" s="17" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C43" s="18" t="n"/>
       <c r="D43" s="18" t="n"/>
@@ -1682,9 +1840,9 @@
         <v/>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="21" customHeight="1">
       <c r="B44" s="17" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C44" s="18" t="n"/>
       <c r="D44" s="18" t="n"/>
@@ -1711,9 +1869,9 @@
         <v/>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="21" customHeight="1">
       <c r="B45" s="17" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C45" s="18" t="n"/>
       <c r="D45" s="18" t="n"/>
@@ -1740,9 +1898,9 @@
         <v/>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="21" customHeight="1">
       <c r="B46" s="17" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C46" s="18" t="n"/>
       <c r="D46" s="18" t="n"/>
@@ -1769,9 +1927,9 @@
         <v/>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="21" customHeight="1">
       <c r="B47" s="17" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C47" s="18" t="n"/>
       <c r="D47" s="18" t="n"/>
@@ -1798,9 +1956,9 @@
         <v/>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="21" customHeight="1">
       <c r="B48" s="17" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C48" s="18" t="n"/>
       <c r="D48" s="18" t="n"/>
@@ -1827,9 +1985,9 @@
         <v/>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="21" customHeight="1">
       <c r="B49" s="17" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C49" s="18" t="n"/>
       <c r="D49" s="18" t="n"/>
@@ -1856,9 +2014,9 @@
         <v/>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="21" customHeight="1">
       <c r="B50" s="17" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C50" s="18" t="n"/>
       <c r="D50" s="18" t="n"/>
@@ -1885,9 +2043,9 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="21" customHeight="1">
       <c r="B51" s="17" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C51" s="18" t="n"/>
       <c r="D51" s="18" t="n"/>
@@ -1914,9 +2072,9 @@
         <v/>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="21" customHeight="1">
       <c r="B52" s="17" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C52" s="18" t="n"/>
       <c r="D52" s="18" t="n"/>
@@ -1943,9 +2101,9 @@
         <v/>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="21" customHeight="1">
       <c r="B53" s="17" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C53" s="18" t="n"/>
       <c r="D53" s="18" t="n"/>
@@ -1972,9 +2130,9 @@
         <v/>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="21" customHeight="1">
       <c r="B54" s="17" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C54" s="18" t="n"/>
       <c r="D54" s="18" t="n"/>
@@ -2001,9 +2159,9 @@
         <v/>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="21" customHeight="1">
       <c r="B55" s="17" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C55" s="18" t="n"/>
       <c r="D55" s="18" t="n"/>
@@ -2030,9 +2188,9 @@
         <v/>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="21" customHeight="1">
       <c r="B56" s="17" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C56" s="18" t="n"/>
       <c r="D56" s="18" t="n"/>
@@ -2059,9 +2217,9 @@
         <v/>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="21" customHeight="1">
       <c r="B57" s="17" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C57" s="18" t="n"/>
       <c r="D57" s="18" t="n"/>
@@ -2088,9 +2246,9 @@
         <v/>
       </c>
     </row>
-    <row r="58">
+    <row r="58" ht="21" customHeight="1">
       <c r="B58" s="17" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C58" s="18" t="n"/>
       <c r="D58" s="18" t="n"/>
@@ -2117,9 +2275,9 @@
         <v/>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="21" customHeight="1">
       <c r="B59" s="17" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C59" s="18" t="n"/>
       <c r="D59" s="18" t="n"/>
@@ -2146,9 +2304,9 @@
         <v/>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="21" customHeight="1">
       <c r="B60" s="17" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C60" s="18" t="n"/>
       <c r="D60" s="18" t="n"/>
@@ -2175,9 +2333,9 @@
         <v/>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="21" customHeight="1">
       <c r="B61" s="17" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C61" s="18" t="n"/>
       <c r="D61" s="18" t="n"/>
@@ -2204,9 +2362,9 @@
         <v/>
       </c>
     </row>
-    <row r="62">
+    <row r="62" ht="21" customHeight="1">
       <c r="B62" s="17" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C62" s="18" t="n"/>
       <c r="D62" s="18" t="n"/>
@@ -2233,9 +2391,9 @@
         <v/>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="21" customHeight="1">
       <c r="B63" s="17" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C63" s="18" t="n"/>
       <c r="D63" s="18" t="n"/>
@@ -2262,9 +2420,9 @@
         <v/>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="21" customHeight="1">
       <c r="B64" s="17" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C64" s="18" t="n"/>
       <c r="D64" s="18" t="n"/>
@@ -2291,9 +2449,9 @@
         <v/>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="21" customHeight="1">
       <c r="B65" s="17" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C65" s="18" t="n"/>
       <c r="D65" s="18" t="n"/>
@@ -2320,9 +2478,9 @@
         <v/>
       </c>
     </row>
-    <row r="66">
+    <row r="66" ht="21" customHeight="1">
       <c r="B66" s="17" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C66" s="18" t="n"/>
       <c r="D66" s="18" t="n"/>
@@ -2349,9 +2507,9 @@
         <v/>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="21" customHeight="1">
       <c r="B67" s="17" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C67" s="18" t="n"/>
       <c r="D67" s="18" t="n"/>
@@ -2378,9 +2536,9 @@
         <v/>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="21" customHeight="1">
       <c r="B68" s="17" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C68" s="18" t="n"/>
       <c r="D68" s="18" t="n"/>
@@ -2407,9 +2565,9 @@
         <v/>
       </c>
     </row>
-    <row r="69">
+    <row r="69" ht="21" customHeight="1">
       <c r="B69" s="17" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C69" s="18" t="n"/>
       <c r="D69" s="18" t="n"/>
@@ -2436,9 +2594,9 @@
         <v/>
       </c>
     </row>
-    <row r="70">
+    <row r="70" ht="21" customHeight="1">
       <c r="B70" s="17" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C70" s="18" t="n"/>
       <c r="D70" s="18" t="n"/>
@@ -2465,9 +2623,9 @@
         <v/>
       </c>
     </row>
-    <row r="71">
+    <row r="71" ht="21" customHeight="1">
       <c r="B71" s="17" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C71" s="18" t="n"/>
       <c r="D71" s="18" t="n"/>
@@ -2494,9 +2652,9 @@
         <v/>
       </c>
     </row>
-    <row r="72">
+    <row r="72" ht="21" customHeight="1">
       <c r="B72" s="17" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C72" s="18" t="n"/>
       <c r="D72" s="18" t="n"/>
@@ -2523,9 +2681,9 @@
         <v/>
       </c>
     </row>
-    <row r="73">
+    <row r="73" ht="21" customHeight="1">
       <c r="B73" s="17" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C73" s="18" t="n"/>
       <c r="D73" s="18" t="n"/>
@@ -2552,9 +2710,9 @@
         <v/>
       </c>
     </row>
-    <row r="74">
+    <row r="74" ht="21" customHeight="1">
       <c r="B74" s="17" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C74" s="18" t="n"/>
       <c r="D74" s="18" t="n"/>
@@ -2581,9 +2739,9 @@
         <v/>
       </c>
     </row>
-    <row r="75">
+    <row r="75" ht="21" customHeight="1">
       <c r="B75" s="17" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C75" s="18" t="n"/>
       <c r="D75" s="18" t="n"/>
@@ -2610,9 +2768,9 @@
         <v/>
       </c>
     </row>
-    <row r="76">
+    <row r="76" ht="21" customHeight="1">
       <c r="B76" s="17" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C76" s="18" t="n"/>
       <c r="D76" s="18" t="n"/>
@@ -2639,9 +2797,9 @@
         <v/>
       </c>
     </row>
-    <row r="77">
+    <row r="77" ht="21" customHeight="1">
       <c r="B77" s="17" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C77" s="18" t="n"/>
       <c r="D77" s="18" t="n"/>
@@ -2668,9 +2826,9 @@
         <v/>
       </c>
     </row>
-    <row r="78">
+    <row r="78" ht="21" customHeight="1">
       <c r="B78" s="17" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C78" s="18" t="n"/>
       <c r="D78" s="18" t="n"/>
@@ -2697,9 +2855,9 @@
         <v/>
       </c>
     </row>
-    <row r="79">
+    <row r="79" ht="21" customHeight="1">
       <c r="B79" s="17" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C79" s="18" t="n"/>
       <c r="D79" s="18" t="n"/>
@@ -2726,9 +2884,9 @@
         <v/>
       </c>
     </row>
-    <row r="80">
+    <row r="80" ht="21" customHeight="1">
       <c r="B80" s="17" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C80" s="18" t="n"/>
       <c r="D80" s="18" t="n"/>
@@ -2755,9 +2913,9 @@
         <v/>
       </c>
     </row>
-    <row r="81">
+    <row r="81" ht="21" customHeight="1">
       <c r="B81" s="17" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C81" s="18" t="n"/>
       <c r="D81" s="18" t="n"/>
@@ -2784,9 +2942,9 @@
         <v/>
       </c>
     </row>
-    <row r="82">
+    <row r="82" ht="21" customHeight="1">
       <c r="B82" s="17" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C82" s="18" t="n"/>
       <c r="D82" s="18" t="n"/>
@@ -2813,9 +2971,9 @@
         <v/>
       </c>
     </row>
-    <row r="83">
+    <row r="83" ht="21" customHeight="1">
       <c r="B83" s="17" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C83" s="18" t="n"/>
       <c r="D83" s="18" t="n"/>
@@ -2842,9 +3000,9 @@
         <v/>
       </c>
     </row>
-    <row r="84">
+    <row r="84" ht="21" customHeight="1">
       <c r="B84" s="17" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C84" s="18" t="n"/>
       <c r="D84" s="18" t="n"/>
@@ -2871,9 +3029,9 @@
         <v/>
       </c>
     </row>
-    <row r="85">
+    <row r="85" ht="21" customHeight="1">
       <c r="B85" s="17" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C85" s="18" t="n"/>
       <c r="D85" s="18" t="n"/>
@@ -2900,9 +3058,9 @@
         <v/>
       </c>
     </row>
-    <row r="86">
+    <row r="86" ht="21" customHeight="1">
       <c r="B86" s="17" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C86" s="18" t="n"/>
       <c r="D86" s="18" t="n"/>
@@ -2929,9 +3087,9 @@
         <v/>
       </c>
     </row>
-    <row r="87">
+    <row r="87" ht="21" customHeight="1">
       <c r="B87" s="17" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C87" s="18" t="n"/>
       <c r="D87" s="18" t="n"/>
@@ -2958,9 +3116,9 @@
         <v/>
       </c>
     </row>
-    <row r="88">
+    <row r="88" ht="21" customHeight="1">
       <c r="B88" s="17" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C88" s="18" t="n"/>
       <c r="D88" s="18" t="n"/>
@@ -2987,9 +3145,9 @@
         <v/>
       </c>
     </row>
-    <row r="89">
+    <row r="89" ht="21" customHeight="1">
       <c r="B89" s="17" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C89" s="18" t="n"/>
       <c r="D89" s="18" t="n"/>
@@ -3016,9 +3174,9 @@
         <v/>
       </c>
     </row>
-    <row r="90">
+    <row r="90" ht="21" customHeight="1">
       <c r="B90" s="17" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C90" s="18" t="n"/>
       <c r="D90" s="18" t="n"/>
@@ -3045,9 +3203,9 @@
         <v/>
       </c>
     </row>
-    <row r="91">
+    <row r="91" ht="21" customHeight="1">
       <c r="B91" s="17" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C91" s="18" t="n"/>
       <c r="D91" s="18" t="n"/>
@@ -3074,9 +3232,9 @@
         <v/>
       </c>
     </row>
-    <row r="92">
+    <row r="92" ht="21" customHeight="1">
       <c r="B92" s="17" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C92" s="18" t="n"/>
       <c r="D92" s="18" t="n"/>
@@ -3103,9 +3261,9 @@
         <v/>
       </c>
     </row>
-    <row r="93">
+    <row r="93" ht="21" customHeight="1">
       <c r="B93" s="17" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C93" s="18" t="n"/>
       <c r="D93" s="18" t="n"/>
@@ -3132,9 +3290,9 @@
         <v/>
       </c>
     </row>
-    <row r="94">
+    <row r="94" ht="21" customHeight="1">
       <c r="B94" s="17" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C94" s="18" t="n"/>
       <c r="D94" s="18" t="n"/>
@@ -3161,9 +3319,9 @@
         <v/>
       </c>
     </row>
-    <row r="95">
+    <row r="95" ht="21" customHeight="1">
       <c r="B95" s="17" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C95" s="18" t="n"/>
       <c r="D95" s="18" t="n"/>
@@ -3190,9 +3348,9 @@
         <v/>
       </c>
     </row>
-    <row r="96">
+    <row r="96" ht="21" customHeight="1">
       <c r="B96" s="17" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C96" s="18" t="n"/>
       <c r="D96" s="18" t="n"/>
@@ -3219,9 +3377,9 @@
         <v/>
       </c>
     </row>
-    <row r="97">
+    <row r="97" ht="21" customHeight="1">
       <c r="B97" s="17" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C97" s="18" t="n"/>
       <c r="D97" s="18" t="n"/>
@@ -3248,9 +3406,9 @@
         <v/>
       </c>
     </row>
-    <row r="98">
+    <row r="98" ht="21" customHeight="1">
       <c r="B98" s="17" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C98" s="18" t="n"/>
       <c r="D98" s="18" t="n"/>
@@ -3277,9 +3435,9 @@
         <v/>
       </c>
     </row>
-    <row r="99">
+    <row r="99" ht="21" customHeight="1">
       <c r="B99" s="17" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C99" s="18" t="n"/>
       <c r="D99" s="18" t="n"/>
@@ -3306,9 +3464,9 @@
         <v/>
       </c>
     </row>
-    <row r="100">
+    <row r="100" ht="21" customHeight="1">
       <c r="B100" s="17" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C100" s="18" t="n"/>
       <c r="D100" s="18" t="n"/>
@@ -3335,9 +3493,9 @@
         <v/>
       </c>
     </row>
-    <row r="101">
+    <row r="101" ht="21" customHeight="1">
       <c r="B101" s="17" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C101" s="18" t="n"/>
       <c r="D101" s="18" t="n"/>
@@ -3364,9 +3522,9 @@
         <v/>
       </c>
     </row>
-    <row r="102">
+    <row r="102" ht="21" customHeight="1">
       <c r="B102" s="17" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C102" s="18" t="n"/>
       <c r="D102" s="18" t="n"/>
@@ -3393,9 +3551,9 @@
         <v/>
       </c>
     </row>
-    <row r="103">
+    <row r="103" ht="21" customHeight="1">
       <c r="B103" s="17" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C103" s="18" t="n"/>
       <c r="D103" s="18" t="n"/>
@@ -3422,9 +3580,9 @@
         <v/>
       </c>
     </row>
-    <row r="104">
+    <row r="104" ht="21" customHeight="1">
       <c r="B104" s="17" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C104" s="18" t="n"/>
       <c r="D104" s="18" t="n"/>
@@ -3451,9 +3609,9 @@
         <v/>
       </c>
     </row>
-    <row r="105">
+    <row r="105" ht="21" customHeight="1">
       <c r="B105" s="17" t="n">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C105" s="18" t="n"/>
       <c r="D105" s="18" t="n"/>
@@ -3480,9 +3638,9 @@
         <v/>
       </c>
     </row>
-    <row r="106">
+    <row r="106" ht="21" customHeight="1">
       <c r="B106" s="17" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C106" s="18" t="n"/>
       <c r="D106" s="18" t="n"/>
@@ -3509,9 +3667,9 @@
         <v/>
       </c>
     </row>
-    <row r="107">
+    <row r="107" ht="21" customHeight="1">
       <c r="B107" s="17" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C107" s="18" t="n"/>
       <c r="D107" s="18" t="n"/>
@@ -3538,9 +3696,9 @@
         <v/>
       </c>
     </row>
-    <row r="108">
+    <row r="108" ht="21" customHeight="1">
       <c r="B108" s="17" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C108" s="18" t="n"/>
       <c r="D108" s="18" t="n"/>
@@ -3567,9 +3725,9 @@
         <v/>
       </c>
     </row>
-    <row r="109">
+    <row r="109" ht="21" customHeight="1">
       <c r="B109" s="17" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C109" s="18" t="n"/>
       <c r="D109" s="18" t="n"/>
@@ -3596,9 +3754,9 @@
         <v/>
       </c>
     </row>
-    <row r="110">
+    <row r="110" ht="21" customHeight="1">
       <c r="B110" s="17" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C110" s="18" t="n"/>
       <c r="D110" s="18" t="n"/>
@@ -3625,9 +3783,9 @@
         <v/>
       </c>
     </row>
-    <row r="111">
+    <row r="111" ht="21" customHeight="1">
       <c r="B111" s="17" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C111" s="18" t="n"/>
       <c r="D111" s="18" t="n"/>
@@ -3654,9 +3812,9 @@
         <v/>
       </c>
     </row>
-    <row r="112">
+    <row r="112" ht="21" customHeight="1">
       <c r="B112" s="17" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C112" s="18" t="n"/>
       <c r="D112" s="18" t="n"/>
@@ -3683,9 +3841,9 @@
         <v/>
       </c>
     </row>
-    <row r="113">
+    <row r="113" ht="21" customHeight="1">
       <c r="B113" s="17" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C113" s="18" t="n"/>
       <c r="D113" s="18" t="n"/>
@@ -3712,9 +3870,9 @@
         <v/>
       </c>
     </row>
-    <row r="114">
+    <row r="114" ht="21" customHeight="1">
       <c r="B114" s="17" t="n">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C114" s="18" t="n"/>
       <c r="D114" s="18" t="n"/>
@@ -3741,9 +3899,9 @@
         <v/>
       </c>
     </row>
-    <row r="115">
+    <row r="115" ht="21" customHeight="1">
       <c r="B115" s="17" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C115" s="18" t="n"/>
       <c r="D115" s="18" t="n"/>
@@ -3770,9 +3928,9 @@
         <v/>
       </c>
     </row>
-    <row r="116">
+    <row r="116" ht="21" customHeight="1">
       <c r="B116" s="17" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C116" s="18" t="n"/>
       <c r="D116" s="18" t="n"/>
@@ -3799,214 +3957,69 @@
         <v/>
       </c>
     </row>
-    <row r="117">
-      <c r="B117" s="17" t="n">
-        <v>96</v>
-      </c>
-      <c r="C117" s="18" t="n"/>
-      <c r="D117" s="18" t="n"/>
-      <c r="E117" s="19" t="n"/>
-      <c r="F117" s="18" t="n"/>
-      <c r="G117" s="20">
-        <f>IF(AND(D117&lt;&gt;"",I117=""),"⚠ revisar","")</f>
-        <v/>
-      </c>
-      <c r="H117">
-        <f>IF(OR($D$5="",C117=""),"",$D$5&amp;"|"&amp;C117)</f>
-        <v/>
-      </c>
-      <c r="I117">
-        <f>IF(OR(H117="",D117=""),"",IFERROR(MATCH(H117&amp;"|"&amp;D117,Preguntas!$F$2:$F$1000,0),""))</f>
-        <v/>
-      </c>
-      <c r="K117">
-        <f>IF(I117="","",INDEX(Preguntas!$D$2:$D$1000,I117))</f>
-        <v/>
-      </c>
-      <c r="L117">
-        <f>IF(K117="","L_YN","L_"&amp;K117)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="118">
-      <c r="B118" s="17" t="n">
-        <v>97</v>
-      </c>
-      <c r="C118" s="18" t="n"/>
-      <c r="D118" s="18" t="n"/>
-      <c r="E118" s="19" t="n"/>
-      <c r="F118" s="18" t="n"/>
-      <c r="G118" s="20">
-        <f>IF(AND(D118&lt;&gt;"",I118=""),"⚠ revisar","")</f>
-        <v/>
-      </c>
-      <c r="H118">
-        <f>IF(OR($D$5="",C118=""),"",$D$5&amp;"|"&amp;C118)</f>
-        <v/>
-      </c>
-      <c r="I118">
-        <f>IF(OR(H118="",D118=""),"",IFERROR(MATCH(H118&amp;"|"&amp;D118,Preguntas!$F$2:$F$1000,0),""))</f>
-        <v/>
-      </c>
-      <c r="K118">
-        <f>IF(I118="","",INDEX(Preguntas!$D$2:$D$1000,I118))</f>
-        <v/>
-      </c>
-      <c r="L118">
-        <f>IF(K118="","L_YN","L_"&amp;K118)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="119">
-      <c r="B119" s="17" t="n">
-        <v>98</v>
-      </c>
-      <c r="C119" s="18" t="n"/>
-      <c r="D119" s="18" t="n"/>
-      <c r="E119" s="19" t="n"/>
-      <c r="F119" s="18" t="n"/>
-      <c r="G119" s="20">
-        <f>IF(AND(D119&lt;&gt;"",I119=""),"⚠ revisar","")</f>
-        <v/>
-      </c>
-      <c r="H119">
-        <f>IF(OR($D$5="",C119=""),"",$D$5&amp;"|"&amp;C119)</f>
-        <v/>
-      </c>
-      <c r="I119">
-        <f>IF(OR(H119="",D119=""),"",IFERROR(MATCH(H119&amp;"|"&amp;D119,Preguntas!$F$2:$F$1000,0),""))</f>
-        <v/>
-      </c>
-      <c r="K119">
-        <f>IF(I119="","",INDEX(Preguntas!$D$2:$D$1000,I119))</f>
-        <v/>
-      </c>
-      <c r="L119">
-        <f>IF(K119="","L_YN","L_"&amp;K119)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="120">
-      <c r="B120" s="17" t="n">
-        <v>99</v>
-      </c>
-      <c r="C120" s="18" t="n"/>
-      <c r="D120" s="18" t="n"/>
-      <c r="E120" s="19" t="n"/>
-      <c r="F120" s="18" t="n"/>
-      <c r="G120" s="20">
-        <f>IF(AND(D120&lt;&gt;"",I120=""),"⚠ revisar","")</f>
-        <v/>
-      </c>
-      <c r="H120">
-        <f>IF(OR($D$5="",C120=""),"",$D$5&amp;"|"&amp;C120)</f>
-        <v/>
-      </c>
-      <c r="I120">
-        <f>IF(OR(H120="",D120=""),"",IFERROR(MATCH(H120&amp;"|"&amp;D120,Preguntas!$F$2:$F$1000,0),""))</f>
-        <v/>
-      </c>
-      <c r="K120">
-        <f>IF(I120="","",INDEX(Preguntas!$D$2:$D$1000,I120))</f>
-        <v/>
-      </c>
-      <c r="L120">
-        <f>IF(K120="","L_YN","L_"&amp;K120)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="121">
-      <c r="B121" s="17" t="n">
-        <v>100</v>
-      </c>
-      <c r="C121" s="18" t="n"/>
-      <c r="D121" s="18" t="n"/>
-      <c r="E121" s="19" t="n"/>
-      <c r="F121" s="18" t="n"/>
-      <c r="G121" s="20">
-        <f>IF(AND(D121&lt;&gt;"",I121=""),"⚠ revisar","")</f>
-        <v/>
-      </c>
-      <c r="H121">
-        <f>IF(OR($D$5="",C121=""),"",$D$5&amp;"|"&amp;C121)</f>
-        <v/>
-      </c>
-      <c r="I121">
-        <f>IF(OR(H121="",D121=""),"",IFERROR(MATCH(H121&amp;"|"&amp;D121,Preguntas!$F$2:$F$1000,0),""))</f>
-        <v/>
-      </c>
-      <c r="K121">
-        <f>IF(I121="","",INDEX(Preguntas!$D$2:$D$1000,I121))</f>
-        <v/>
-      </c>
-      <c r="L121">
-        <f>IF(K121="","L_YN","L_"&amp;K121)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="24">
     <mergeCell ref="B2:G2"/>
+    <mergeCell ref="F4:G4"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="B14:G14"/>
     <mergeCell ref="B1:G1"/>
+    <mergeCell ref="F5:G12"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="D6:E6"/>
-    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B4:E4"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="D11:E11"/>
-    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D13:E13"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="B13:C13"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B4:G4"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D8:E8"/>
-    <mergeCell ref="B16:G16"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="B18:G18"/>
   </mergeCells>
-  <conditionalFormatting sqref="B16:G20">
+  <conditionalFormatting sqref="F5:G12">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$B16&lt;&gt;""</formula>
+      <formula>AND($F$5&lt;&gt;"",$F$5&lt;&gt;"Sin alertas por ahora.")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>$F$5="Sin alertas por ahora."</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D14">
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>$D$14="ALTA PRIORIDAD"</formula>
+  <conditionalFormatting sqref="D13">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>$D$13="ALTA PRIORIDAD"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E22:E121">
-    <cfRule type="expression" priority="3" dxfId="1" stopIfTrue="1">
-      <formula>OR($E22="Sí",$E22="Funciona")</formula>
+  <conditionalFormatting sqref="E17:E116">
+    <cfRule type="expression" priority="4" dxfId="1" stopIfTrue="1">
+      <formula>OR($E17="Sí",$E17="Funciona")</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
-      <formula>OR($E22="No",$E22="No funciona")</formula>
+    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
+      <formula>OR($E17="No",$E17="No funciona")</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" dxfId="2" stopIfTrue="1">
-      <formula>OR($E22="No sé",$E22="No probado",$E22="No fue posible comprobar")</formula>
+    <cfRule type="expression" priority="6" dxfId="2" stopIfTrue="1">
+      <formula>OR($E17="No sé",$E17="No probado",$E17="No fue posible comprobar")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation sqref="D5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Tipo de equipo" error="Elija un equipo de la lista." promptTitle="Paso 1" prompt="Elija el tipo de equipo." type="list">
       <formula1>=T_EQUIPO</formula1>
     </dataValidation>
-    <dataValidation sqref="C22:C121" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Categoría" error="Primero elija el tipo de equipo (paso 1) y luego una categoría de la lista." promptTitle="Paso 2" prompt="Elija la categoría o falla." type="list">
+    <dataValidation sqref="C17:C116" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Categoría" error="Primero elija el tipo de equipo (paso 1) y luego una categoría de la lista." promptTitle="Paso 2" prompt="Elija la categoría o falla." type="list">
       <formula1>=OFFSET(Listas!$E$2,MATCH($D$5,Listas!$D$2:$D$200,0)-1,0,COUNTIF(Listas!$D$2:$D$200,$D$5),1)</formula1>
     </dataValidation>
-    <dataValidation sqref="D22:D121" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pregunta" error="Primero elija la categoría (paso 2) y luego una pregunta de la lista." promptTitle="Paso 3" prompt="Elija la pregunta." type="list">
-      <formula1>=OFFSET(Preguntas!$C$2,MATCH($D$5&amp;"|"&amp;$C22,Preguntas!$E$2:$E$1000,0)-1,0,COUNTIF(Preguntas!$E$2:$E$1000,$D$5&amp;"|"&amp;$C22),1)</formula1>
+    <dataValidation sqref="D17:D116" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pregunta" error="Primero elija la categoría (paso 2) y luego una pregunta de la lista." promptTitle="Paso 3" prompt="Elija la pregunta." type="list">
+      <formula1>=OFFSET(Preguntas!$C$2,MATCH($D$5&amp;"|"&amp;$C17,Preguntas!$E$2:$E$1000,0)-1,0,COUNTIF(Preguntas!$E$2:$E$1000,$D$5&amp;"|"&amp;$C17),1)</formula1>
     </dataValidation>
-    <dataValidation sqref="E22:E121" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Paso 4" prompt="Elija la respuesta (solo la contraseña se escribe)." type="list">
-      <formula1>=INDIRECT("L_"&amp;IFERROR(INDEX(Preguntas!$D$2:$D$1000,MATCH($D$5&amp;"|"&amp;$C22&amp;"|"&amp;$D22,Preguntas!$F$2:$F$1000,0)),"YN"))</formula1>
+    <dataValidation sqref="E17:E116" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Paso 4" prompt="Elija la respuesta (solo la contraseña se escribe)." type="list">
+      <formula1>=INDIRECT("L_"&amp;IFERROR(INDEX(Preguntas!$D$2:$D$1000,MATCH($D$5&amp;"|"&amp;$C17&amp;"|"&amp;$D17,Preguntas!$F$2:$F$1000,0)),"YN"))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>